<commit_message>
add new annotations from OneDrive
</commit_message>
<xml_diff>
--- a/annotations/W-Act1Sce3.xlsx
+++ b/annotations/W-Act1Sce3.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr dateCompatibility="0" filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E531D109-74C4-4128-92BF-A1AE669B7C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29905"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="2029" documentId="11_7C2C12AEA2420AA7B3FDF94C9B4AEE27579504A0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EAE7DFB-D71B-4B21-BA5D-4F757D9360FE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="1" xr2:uid="{087A1B5B-7B97-4327-AC94-7D0ECF997B43}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28560" windowHeight="13545" firstSheet="1" activeTab="1" xr2:uid="{087A1B5B-7B97-4327-AC94-7D0ECF997B43}"/>
   </bookViews>
   <sheets>
     <sheet name="A1S3 - général" sheetId="1" r:id="rId1"/>
@@ -13,9 +13,6 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
-      <x14:workbookPr/>
-    </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
@@ -35,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="557" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="306">
   <si>
     <t>Code</t>
   </si>
@@ -1297,8 +1294,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1423,37 +1420,37 @@
   </fills>
   <borders count="11">
     <border>
-      <start/>
-      <end/>
+      <left/>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <start style="thin">
-        <color rgb="FF000000"/>
-      </start>
-      <end/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <start style="thin">
-        <color rgb="FF000000"/>
-      </start>
-      <end style="thin">
-        <color rgb="FF000000"/>
-      </end>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <start style="thin">
-        <color rgb="FF000000"/>
-      </start>
-      <end/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -1463,12 +1460,12 @@
       <diagonal/>
     </border>
     <border>
-      <start style="thin">
-        <color rgb="FF000000"/>
-      </start>
-      <end style="thin">
-        <color rgb="FF000000"/>
-      </end>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -1478,10 +1475,10 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end style="thin">
-        <color rgb="FF000000"/>
-      </end>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -1491,10 +1488,10 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end style="thin">
-        <color rgb="FF000000"/>
-      </end>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -1502,17 +1499,17 @@
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end style="thin">
-        <color rgb="FF000000"/>
-      </end>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <start/>
-      <end/>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -1522,12 +1519,12 @@
       <diagonal/>
     </border>
     <border>
-      <start style="thin">
-        <color rgb="FF000000"/>
-      </start>
-      <end style="thin">
-        <color rgb="FF000000"/>
-      </end>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -1535,10 +1532,10 @@
       <diagonal/>
     </border>
     <border>
-      <start style="thin">
-        <color rgb="FF000000"/>
-      </start>
-      <end/>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -1619,9 +1616,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1631,16 +1625,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1672,7 +1669,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://purl.oclc.org/ooxml/drawingml/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1825,25 +1822,25 @@
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0%">
+            <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110%"/>
-                <a:satMod val="105%"/>
-                <a:tint val="67%"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50%">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105%"/>
-                <a:satMod val="103%"/>
-                <a:tint val="73%"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100%">
+            <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105%"/>
-                <a:satMod val="109%"/>
-                <a:tint val="81%"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1851,25 +1848,25 @@
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0%">
+            <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103%"/>
-                <a:lumMod val="102%"/>
-                <a:tint val="94%"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50%">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110%"/>
-                <a:lumMod val="100%"/>
-                <a:shade val="100%"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100%">
+            <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99%"/>
-                <a:satMod val="120%"/>
-                <a:shade val="78%"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1882,21 +1879,21 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800%"/>
+          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800%"/>
+          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800%"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1910,7 +1907,7 @@
           <a:effectLst>
             <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63%"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -1922,32 +1919,32 @@
         </a:solidFill>
         <a:solidFill>
           <a:schemeClr val="phClr">
-            <a:tint val="95%"/>
-            <a:satMod val="170%"/>
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0%">
+            <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93%"/>
-                <a:satMod val="150%"/>
-                <a:shade val="98%"/>
-                <a:lumMod val="102%"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50%">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="98%"/>
-                <a:satMod val="130%"/>
-                <a:shade val="90%"/>
-                <a:lumMod val="103%"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100%">
+            <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63%"/>
-                <a:satMod val="120%"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1987,9 +1984,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B7EDC20-7B7C-4A7E-972E-FECEFF2E9DC1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B7EDC20-7B7C-4A7E-972E-FECEFF2E9DC1}">
   <dimension ref="A1:R42"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15.75"/>
   <cols>
     <col min="2" max="2" width="11.42578125" style="21"/>
     <col min="3" max="3" width="146.7109375" style="2" customWidth="1"/>
@@ -2002,7 +1999,7 @@
     <col min="13" max="18" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2019,11 +2016,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="27">
+      <c r="B2" s="34">
         <v>68</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -2033,35 +2030,35 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="27"/>
+      <c r="B3" s="34"/>
       <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="31" t="s">
+      <c r="G3" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="27"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="33"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="B4" s="34"/>
       <c r="E4" s="21"/>
-      <c r="G4" s="33" t="s">
+      <c r="G4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
       <c r="K4" s="8" t="s">
         <v>11</v>
       </c>
@@ -2069,23 +2066,23 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="18" customHeight="1">
       <c r="A5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="27">
+      <c r="B5" s="34">
         <v>69</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E5" s="21"/>
-      <c r="G5" s="28" t="s">
+      <c r="G5" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="30"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="29"/>
       <c r="K5" s="9" t="s">
         <v>16</v>
       </c>
@@ -2093,21 +2090,21 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="19.5" customHeight="1">
       <c r="A6" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="27"/>
+      <c r="B6" s="34"/>
       <c r="C6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="21"/>
-      <c r="G6" s="28" t="s">
+      <c r="G6" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="30"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="29"/>
       <c r="K6" s="10" t="s">
         <v>21</v>
       </c>
@@ -2115,15 +2112,15 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B7" s="27"/>
+    <row r="7" spans="1:12">
+      <c r="B7" s="34"/>
       <c r="E7" s="21"/>
-      <c r="G7" s="28" t="s">
+      <c r="G7" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="30"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="29"/>
       <c r="K7" s="11" t="s">
         <v>24</v>
       </c>
@@ -2131,23 +2128,23 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12">
       <c r="A8" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="27">
+      <c r="B8" s="34">
         <v>70</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E8" s="21"/>
-      <c r="G8" s="28" t="s">
+      <c r="G8" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="30"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="29"/>
       <c r="K8" s="12" t="s">
         <v>29</v>
       </c>
@@ -2155,21 +2152,21 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12">
       <c r="A9" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="27"/>
+      <c r="B9" s="34"/>
       <c r="C9" s="2" t="s">
         <v>32</v>
       </c>
       <c r="E9" s="21"/>
-      <c r="G9" s="28" t="s">
+      <c r="G9" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="30"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="29"/>
       <c r="K9" s="13" t="s">
         <v>34</v>
       </c>
@@ -2177,21 +2174,21 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12">
       <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="27"/>
+      <c r="B10" s="34"/>
       <c r="C10" s="2" t="s">
         <v>36</v>
       </c>
       <c r="E10" s="21"/>
-      <c r="G10" s="28" t="s">
+      <c r="G10" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="30"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="29"/>
       <c r="K10" s="14" t="s">
         <v>38</v>
       </c>
@@ -2199,15 +2196,15 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B11" s="27"/>
+    <row r="11" spans="1:12">
+      <c r="B11" s="34"/>
       <c r="E11" s="21"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12">
       <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="34">
         <v>72</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -2218,53 +2215,53 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="27"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12">
+      <c r="B13" s="34"/>
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="27">
+      <c r="B14" s="34">
         <v>73</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="27"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12">
+      <c r="B15" s="34"/>
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="27">
+      <c r="B16" s="34">
         <v>74</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="27"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4">
+      <c r="B17" s="34"/>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
         <v>18</v>
       </c>
-      <c r="B18" s="27">
+      <c r="B18" s="34">
         <v>78</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" ht="20.25" customHeight="1">
       <c r="A19" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="27"/>
+      <c r="B19" s="34"/>
       <c r="C19" s="23" t="s">
         <v>45</v>
       </c>
@@ -2272,32 +2269,32 @@
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="27"/>
+      <c r="B20" s="34"/>
       <c r="C20" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="27"/>
+      <c r="B21" s="34"/>
       <c r="C21" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B22" s="27"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4">
+      <c r="B22" s="34"/>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="27">
+      <c r="B23" s="34">
         <v>80</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -2307,20 +2304,20 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="27"/>
+      <c r="B24" s="34"/>
       <c r="C24" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="27"/>
+      <c r="B25" s="34"/>
       <c r="C25" s="2" t="s">
         <v>53</v>
       </c>
@@ -2328,42 +2325,42 @@
         <v>46</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B26" s="27"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4">
+      <c r="B26" s="34"/>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="27">
+      <c r="B27" s="34">
         <v>81</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B28" s="27"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4">
+      <c r="B28" s="34"/>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>5</v>
       </c>
-      <c r="B29" s="27">
+      <c r="B29" s="34">
         <v>82</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B30" s="27"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4">
+      <c r="B30" s="34"/>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31" t="s">
         <v>18</v>
       </c>
-      <c r="B31" s="27">
+      <c r="B31" s="34">
         <v>90</v>
       </c>
       <c r="C31" s="2" t="s">
@@ -2373,85 +2370,85 @@
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B32" s="27"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4">
+      <c r="B32" s="34"/>
+    </row>
+    <row r="33" spans="1:3">
       <c r="A33" t="s">
         <v>18</v>
       </c>
-      <c r="B33" s="27">
+      <c r="B33" s="34">
         <v>92</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="27"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3">
+      <c r="B34" s="34"/>
+    </row>
+    <row r="35" spans="1:3">
       <c r="A35" t="s">
         <v>18</v>
       </c>
-      <c r="B35" s="27">
+      <c r="B35" s="34">
         <v>94</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3">
       <c r="A36" t="s">
         <v>26</v>
       </c>
-      <c r="B36" s="27"/>
+      <c r="B36" s="34"/>
       <c r="C36" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B37" s="27"/>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3">
+      <c r="B37" s="34"/>
+    </row>
+    <row r="38" spans="1:3">
       <c r="A38" t="s">
         <v>13</v>
       </c>
-      <c r="B38" s="27">
+      <c r="B38" s="34">
         <v>98</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B39" s="27"/>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3">
+      <c r="B39" s="34"/>
+    </row>
+    <row r="40" spans="1:3">
       <c r="A40" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="27">
+      <c r="B40" s="34">
         <v>109</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3">
       <c r="A41" t="s">
         <v>18</v>
       </c>
-      <c r="B41" s="27"/>
+      <c r="B41" s="34"/>
       <c r="C41" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3">
       <c r="A42" t="s">
         <v>18</v>
       </c>
-      <c r="B42" s="27"/>
+      <c r="B42" s="34"/>
       <c r="C42" s="2" t="s">
         <v>64</v>
       </c>
@@ -2473,12 +2470,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9AB9CF3-2A5A-48E8-AAD8-D77A773B0227}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9AB9CF3-2A5A-48E8-AAD8-D77A773B0227}">
   <dimension ref="A1:R223"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="1"/>
-    <col min="2" max="2" width="11.42578125" style="27"/>
+    <col min="2" max="2" width="11.42578125" style="34"/>
     <col min="3" max="3" width="102.5703125" style="2" customWidth="1"/>
     <col min="4" max="4" width="44.140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="39" style="21" bestFit="1" customWidth="1"/>
@@ -2490,7 +2487,7 @@
     <col min="13" max="18" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2507,11 +2504,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="27">
+      <c r="B2" s="34">
         <v>325</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -2524,41 +2521,41 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="27">
+      <c r="B3" s="34">
         <v>325</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="G3" s="31" t="s">
+      <c r="G3" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="33"/>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="27">
+      <c r="B4" s="34">
         <v>325</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="G4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
       <c r="K4" s="8" t="s">
         <v>11</v>
       </c>
@@ -2566,11 +2563,11 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12">
       <c r="A5" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="34" t="s">
         <v>73</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -2583,22 +2580,22 @@
       <c r="K5" s="26"/>
       <c r="L5" s="7"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12">
       <c r="A6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="27">
+      <c r="B6" s="34">
         <v>326</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="G6" s="28" t="s">
+      <c r="G6" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="30"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="29"/>
       <c r="K6" s="9" t="s">
         <v>16</v>
       </c>
@@ -2606,11 +2603,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="34" t="s">
         <v>76</v>
       </c>
       <c r="C7" s="2" t="s">
@@ -2619,12 +2616,12 @@
       <c r="D7" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G7" s="28" t="s">
+      <c r="G7" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="29"/>
-      <c r="I7" s="29"/>
-      <c r="J7" s="30"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="29"/>
       <c r="K7" s="10" t="s">
         <v>21</v>
       </c>
@@ -2632,22 +2629,22 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12">
       <c r="A8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="27">
+      <c r="B8" s="34">
         <v>328</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="G8" s="28" t="s">
+      <c r="G8" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="29"/>
-      <c r="I8" s="29"/>
-      <c r="J8" s="30"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="29"/>
       <c r="K8" s="11" t="s">
         <v>24</v>
       </c>
@@ -2655,19 +2652,19 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="27">
+    <row r="9" spans="1:12">
+      <c r="B9" s="34">
         <v>328</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G9" s="28" t="s">
+      <c r="G9" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="H9" s="29"/>
-      <c r="I9" s="29"/>
-      <c r="J9" s="30"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="29"/>
       <c r="K9" s="12" t="s">
         <v>29</v>
       </c>
@@ -2675,22 +2672,22 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="27">
+      <c r="B10" s="34">
         <v>329</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="G10" s="28" t="s">
+      <c r="G10" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="30"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="29"/>
       <c r="K10" s="13" t="s">
         <v>34</v>
       </c>
@@ -2698,22 +2695,22 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12">
       <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="27">
+      <c r="B11" s="34">
         <v>329</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="G11" s="28" t="s">
+      <c r="G11" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="29"/>
-      <c r="I11" s="29"/>
-      <c r="J11" s="30"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="29"/>
       <c r="K11" s="14" t="s">
         <v>38</v>
       </c>
@@ -2721,11 +2718,11 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12">
       <c r="A13" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="27">
+      <c r="B13" s="34">
         <v>330</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -2735,88 +2732,88 @@
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12">
       <c r="A14" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B14" s="27">
+      <c r="B14" s="34">
         <v>332</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12">
       <c r="A16" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="27">
+      <c r="B16" s="34">
         <v>334</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4">
       <c r="A17" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="27">
+      <c r="B17" s="34">
         <v>334</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4">
       <c r="A18" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="27">
+      <c r="B18" s="34">
         <v>334</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4">
       <c r="A19" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="34" t="s">
         <v>89</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4">
       <c r="A20" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="27">
+      <c r="B20" s="34">
         <v>337</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4">
       <c r="A21" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B21" s="27">
+      <c r="B21" s="34">
         <v>339</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4">
       <c r="A23" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="27">
+      <c r="B23" s="34">
         <v>342</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -2826,338 +2823,338 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4">
       <c r="A25" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B25" s="27">
+      <c r="B25" s="34">
         <v>345</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4">
       <c r="A27" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B27" s="27">
+      <c r="B27" s="34">
         <v>346</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4">
       <c r="A28" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B28" s="27">
+      <c r="B28" s="34">
         <v>346</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4">
       <c r="A29" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="27">
+      <c r="B29" s="34">
         <v>346</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B30" s="27">
+    <row r="30" spans="1:4">
+      <c r="B30" s="34">
         <v>350</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4">
       <c r="A31" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B31" s="27">
+      <c r="B31" s="34">
         <v>350</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4">
       <c r="A32" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B32" s="27" t="s">
+      <c r="B32" s="34" t="s">
         <v>100</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3">
       <c r="A34" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B34" s="27" t="s">
+      <c r="B34" s="34" t="s">
         <v>102</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3">
       <c r="A36" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B36" s="27" t="s">
+      <c r="B36" s="34" t="s">
         <v>104</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3">
       <c r="A37" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B37" s="27">
+      <c r="B37" s="34">
         <v>356</v>
       </c>
       <c r="C37" s="23" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3">
       <c r="A38" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B38" s="27">
+      <c r="B38" s="34">
         <v>256</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3">
       <c r="A39" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="27">
+      <c r="B39" s="34">
         <v>360</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3">
       <c r="A40" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B40" s="27">
+      <c r="B40" s="34">
         <v>362</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3">
       <c r="A41" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B41" s="27">
+      <c r="B41" s="34">
         <v>362</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3">
       <c r="A42" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B42" s="27">
+      <c r="B42" s="34">
         <v>362</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3">
       <c r="A43" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B43" s="27">
+      <c r="B43" s="34">
         <v>362</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3">
       <c r="A45" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B45" s="27">
+      <c r="B45" s="34">
         <v>363</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3">
       <c r="A46" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B46" s="27">
+      <c r="B46" s="34">
         <v>363</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3">
       <c r="A47" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B47" s="27">
+      <c r="B47" s="34">
         <v>363</v>
       </c>
       <c r="C47" s="23" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3">
       <c r="A48" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B48" s="27">
+      <c r="B48" s="34">
         <v>363</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4">
       <c r="A49" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B49" s="27">
+      <c r="B49" s="34">
         <v>364</v>
       </c>
       <c r="C49" s="23" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4">
       <c r="A50" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B50" s="27" t="s">
+      <c r="B50" s="34" t="s">
         <v>118</v>
       </c>
       <c r="C50" s="23" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4">
       <c r="A51" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B51" s="27">
+      <c r="B51" s="34">
         <v>365</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4">
       <c r="A52" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B52" s="27">
+      <c r="B52" s="34">
         <v>365</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4">
       <c r="A53" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B53" s="27">
+      <c r="B53" s="34">
         <v>365</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4">
       <c r="A55" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B55" s="27">
+      <c r="B55" s="34">
         <v>366</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4">
       <c r="A56" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B56" s="27">
+      <c r="B56" s="34">
         <v>367</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4">
       <c r="A57" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B57" s="27">
+      <c r="B57" s="34">
         <v>368</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4">
       <c r="A58" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B58" s="27">
+      <c r="B58" s="34">
         <v>368</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4">
       <c r="A59" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B59" s="27">
+      <c r="B59" s="34">
         <v>369</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4">
       <c r="A60" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B60" s="27">
+      <c r="B60" s="34">
         <v>369</v>
       </c>
       <c r="C60" s="2" t="s">
@@ -3167,183 +3164,183 @@
         <v>78</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4">
       <c r="A62" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B62" s="27">
+      <c r="B62" s="34">
         <v>370</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4">
       <c r="A63" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B63" s="27">
+      <c r="B63" s="34">
         <v>370</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4">
       <c r="A64" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B64" s="27">
+      <c r="B64" s="34">
         <v>370</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4">
       <c r="A65" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B65" s="27">
+      <c r="B65" s="34">
         <v>370</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4">
       <c r="A66" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B66" s="27">
+      <c r="B66" s="34">
         <v>370</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4">
       <c r="A67" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B67" s="27">
+      <c r="B67" s="34">
         <v>371</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4">
       <c r="A68" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B68" s="27">
+      <c r="B68" s="34">
         <v>372</v>
       </c>
       <c r="C68" s="2" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4">
       <c r="A69" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B69" s="27">
+      <c r="B69" s="34">
         <v>372</v>
       </c>
       <c r="C69" s="23" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4">
       <c r="A70" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B70" s="27">
+      <c r="B70" s="34">
         <v>372</v>
       </c>
       <c r="C70" s="23" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4">
       <c r="A71" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B71" s="27">
+      <c r="B71" s="34">
         <v>373</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4">
       <c r="A72" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B72" s="27">
+      <c r="B72" s="34">
         <v>373</v>
       </c>
       <c r="C72" s="2" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4">
       <c r="A73" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B73" s="27" t="s">
+      <c r="B73" s="34" t="s">
         <v>140</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4">
       <c r="A74" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B74" s="27">
+      <c r="B74" s="34">
         <v>374</v>
       </c>
       <c r="C74" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4">
       <c r="A76" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B76" s="27">
+      <c r="B76" s="34">
         <v>375</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4">
       <c r="A77" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B77" s="27">
+      <c r="B77" s="34">
         <v>375</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4">
       <c r="A78" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B78" s="27" t="s">
+      <c r="B78" s="34" t="s">
         <v>145</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4">
       <c r="A79" s="1" t="s">
         <v>26</v>
       </c>
@@ -3351,11 +3348,11 @@
         <v>147</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4">
       <c r="A80" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B80" s="27">
+      <c r="B80" s="34">
         <v>378</v>
       </c>
       <c r="C80" s="2" t="s">
@@ -3365,66 +3362,66 @@
         <v>149</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4">
       <c r="A81" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B81" s="27">
+      <c r="B81" s="34">
         <v>379</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4">
       <c r="A83" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B83" s="27">
+      <c r="B83" s="34">
         <v>380</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4">
       <c r="A84" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B84" s="27">
+      <c r="B84" s="34">
         <v>380</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4">
       <c r="A85" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B85" s="27" t="s">
+      <c r="B85" s="34" t="s">
         <v>153</v>
       </c>
       <c r="C85" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4">
       <c r="A86" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B86" s="27">
+      <c r="B86" s="34">
         <v>380</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4">
       <c r="A87" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B87" s="27" t="s">
+      <c r="B87" s="34" t="s">
         <v>156</v>
       </c>
       <c r="C87" s="2" t="s">
@@ -3434,22 +3431,22 @@
         <v>158</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4">
       <c r="A88" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B88" s="27" t="s">
+      <c r="B88" s="34" t="s">
         <v>156</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4">
       <c r="A89" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B89" s="27">
+      <c r="B89" s="34">
         <v>385</v>
       </c>
       <c r="C89" s="2" t="s">
@@ -3459,66 +3456,66 @@
         <v>46</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4">
       <c r="A90" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B90" s="27">
+      <c r="B90" s="34">
         <v>385</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4">
       <c r="A91" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B91" s="27" t="s">
+      <c r="B91" s="34" t="s">
         <v>162</v>
       </c>
       <c r="C91" s="2" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4">
       <c r="A92" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B92" s="27">
+      <c r="B92" s="34">
         <v>388</v>
       </c>
       <c r="C92" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4">
       <c r="A93" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B93" s="27">
+      <c r="B93" s="34">
         <v>388</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4">
       <c r="A94" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B94" s="27">
+      <c r="B94" s="34">
         <v>388</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4">
       <c r="A95" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B95" s="27">
+      <c r="B95" s="34">
         <v>388</v>
       </c>
       <c r="C95" s="2" t="s">
@@ -3528,132 +3525,132 @@
         <v>168</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4">
       <c r="A97" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B97" s="27">
+      <c r="B97" s="34">
         <v>392</v>
       </c>
       <c r="C97" s="2" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4">
       <c r="A98" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B98" s="27">
+      <c r="B98" s="34">
         <v>392</v>
       </c>
       <c r="C98" s="2" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4">
       <c r="A99" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B99" s="27">
+      <c r="B99" s="34">
         <v>392</v>
       </c>
       <c r="C99" s="2" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4">
       <c r="A101" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B101" s="27">
+      <c r="B101" s="34">
         <v>394</v>
       </c>
       <c r="C101" s="2" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4">
       <c r="A102" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B102" s="27">
+      <c r="B102" s="34">
         <v>396</v>
       </c>
       <c r="C102" s="2" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4">
       <c r="A103" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B103" s="27" t="s">
+      <c r="B103" s="34" t="s">
         <v>174</v>
       </c>
       <c r="C103" s="2" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4">
       <c r="A104" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B104" s="27" t="s">
+      <c r="B104" s="34" t="s">
         <v>174</v>
       </c>
       <c r="C104" s="2" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4">
       <c r="A105" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B105" s="27">
+      <c r="B105" s="34">
         <v>396</v>
       </c>
       <c r="C105" s="2" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4">
       <c r="A106" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B106" s="27">
+      <c r="B106" s="34">
         <v>396</v>
       </c>
       <c r="C106" s="2" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4">
       <c r="A107" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B107" s="27" t="s">
+      <c r="B107" s="34" t="s">
         <v>174</v>
       </c>
       <c r="C107" s="2" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4">
       <c r="A109" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B109" s="27">
+      <c r="B109" s="34">
         <v>398</v>
       </c>
       <c r="C109" s="2" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4">
       <c r="A110" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B110" s="27">
+      <c r="B110" s="34">
         <v>398</v>
       </c>
       <c r="C110" s="2" t="s">
@@ -3663,66 +3660,66 @@
         <v>181</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4">
       <c r="A111" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B111" s="27">
+      <c r="B111" s="34">
         <v>399</v>
       </c>
       <c r="C111" s="2" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4">
       <c r="A112" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B112" s="27" t="s">
+      <c r="B112" s="34" t="s">
         <v>183</v>
       </c>
       <c r="C112" s="2" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5">
       <c r="A113" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B113" s="27">
+      <c r="B113" s="34">
         <v>399</v>
       </c>
       <c r="C113" s="2" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5">
       <c r="A114" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B114" s="27" t="s">
+      <c r="B114" s="34" t="s">
         <v>186</v>
       </c>
       <c r="C114" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5">
       <c r="A115" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B115" s="27">
+      <c r="B115" s="34">
         <v>400</v>
       </c>
       <c r="C115" s="2" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5">
       <c r="A116" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B116" s="27">
+      <c r="B116" s="34">
         <v>400</v>
       </c>
       <c r="C116" s="2" t="s">
@@ -3732,110 +3729,110 @@
         <v>190</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5">
       <c r="A117" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B117" s="27">
+      <c r="B117" s="34">
         <v>403</v>
       </c>
       <c r="C117" s="2" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5">
       <c r="A118" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B118" s="27">
+      <c r="B118" s="34">
         <v>403</v>
       </c>
       <c r="C118" s="2" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5">
       <c r="A119" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B119" s="27" t="s">
+      <c r="B119" s="34" t="s">
         <v>193</v>
       </c>
       <c r="C119" s="2" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5">
       <c r="A120" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B120" s="27">
+      <c r="B120" s="34">
         <v>403</v>
       </c>
       <c r="C120" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5">
       <c r="A121" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B121" s="27">
+      <c r="B121" s="34">
         <v>405</v>
       </c>
       <c r="C121" s="2" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5">
       <c r="A122" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="B122" s="27">
+      <c r="B122" s="34">
         <v>407</v>
       </c>
       <c r="C122" s="2" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5">
       <c r="A123" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B123" s="27" t="s">
+      <c r="B123" s="34" t="s">
         <v>199</v>
       </c>
       <c r="C123" s="2" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5">
       <c r="A124" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B124" s="27" t="s">
+      <c r="B124" s="34" t="s">
         <v>201</v>
       </c>
       <c r="C124" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5">
       <c r="A125" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B125" s="27">
+      <c r="B125" s="34">
         <v>412</v>
       </c>
       <c r="C125" s="2" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5">
       <c r="A126" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B126" s="27">
+      <c r="B126" s="34">
         <v>412</v>
       </c>
       <c r="C126" s="2" t="s">
@@ -3848,22 +3845,22 @@
         <v>205</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5">
       <c r="A127" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B127" s="27">
+      <c r="B127" s="34">
         <v>412</v>
       </c>
       <c r="C127" s="2" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5">
       <c r="A128" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B128" s="27">
+      <c r="B128" s="34">
         <v>415</v>
       </c>
       <c r="C128" s="2" t="s">
@@ -3873,66 +3870,66 @@
         <v>208</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4">
       <c r="A129" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B129" s="27">
+      <c r="B129" s="34">
         <v>415</v>
       </c>
       <c r="C129" s="2" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4">
       <c r="A131" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B131" s="27">
+      <c r="B131" s="34">
         <v>417</v>
       </c>
       <c r="C131" s="2" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4">
       <c r="A132" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B132" s="27">
+      <c r="B132" s="34">
         <v>417</v>
       </c>
       <c r="C132" s="2" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4">
       <c r="A133" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B133" s="27" t="s">
+      <c r="B133" s="34" t="s">
         <v>212</v>
       </c>
       <c r="C133" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4">
       <c r="A134" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B134" s="27">
+      <c r="B134" s="34">
         <v>419</v>
       </c>
       <c r="C134" s="2" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4">
       <c r="A135" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B135" s="27">
+      <c r="B135" s="34">
         <v>419</v>
       </c>
       <c r="C135" s="2" t="s">
@@ -3942,176 +3939,176 @@
         <v>215</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4">
       <c r="A136" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B136" s="27">
+      <c r="B136" s="34">
         <v>422</v>
       </c>
       <c r="C136" s="2" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:4">
       <c r="A137" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B137" s="27">
+      <c r="B137" s="34">
         <v>422</v>
       </c>
       <c r="C137" s="2" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4">
       <c r="A138" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B138" s="27">
+      <c r="B138" s="34">
         <v>422</v>
       </c>
       <c r="C138" s="2" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:4">
       <c r="A139" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B139" s="27">
+      <c r="B139" s="34">
         <v>422</v>
       </c>
       <c r="C139" s="2" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4">
       <c r="A140" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B140" s="27">
+      <c r="B140" s="34">
         <v>424</v>
       </c>
       <c r="D140" s="1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4">
       <c r="A141" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B141" s="27">
+      <c r="B141" s="34">
         <v>425</v>
       </c>
       <c r="C141" s="2" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4">
       <c r="A142" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B142" s="27">
+      <c r="B142" s="34">
         <v>427</v>
       </c>
       <c r="C142" s="23" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4">
       <c r="A143" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B143" s="27">
+      <c r="B143" s="34">
         <v>427</v>
       </c>
       <c r="C143" s="2" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4">
       <c r="A144" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B144" s="27">
+      <c r="B144" s="34">
         <v>428</v>
       </c>
       <c r="C144" s="2" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4">
       <c r="A145" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B145" s="27">
+      <c r="B145" s="34">
         <v>428</v>
       </c>
       <c r="C145" s="2" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4">
       <c r="A146" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B146" s="27">
+      <c r="B146" s="34">
         <v>428</v>
       </c>
       <c r="C146" s="23" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:4">
       <c r="A147" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B147" s="27">
+      <c r="B147" s="34">
         <v>429</v>
       </c>
       <c r="C147" s="2" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:4">
       <c r="A149" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B149" s="27">
+      <c r="B149" s="34">
         <v>430</v>
       </c>
       <c r="C149" s="2" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:4">
       <c r="A150" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B150" s="27">
+      <c r="B150" s="34">
         <v>431</v>
       </c>
       <c r="C150" s="2" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:4">
       <c r="A151" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B151" s="27">
+      <c r="B151" s="34">
         <v>433</v>
       </c>
       <c r="C151" s="23" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4">
       <c r="A152" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B152" s="27">
+      <c r="B152" s="34">
         <v>433</v>
       </c>
       <c r="C152" s="2" t="s">
@@ -4121,99 +4118,99 @@
         <v>233</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:4">
       <c r="A154" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B154" s="27">
+      <c r="B154" s="34">
         <v>435</v>
       </c>
       <c r="C154" s="2" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:4">
       <c r="A155" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B155" s="27">
+      <c r="B155" s="34">
         <v>435</v>
       </c>
       <c r="C155" s="2" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:4">
       <c r="A156" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B156" s="27">
+      <c r="B156" s="34">
         <v>435</v>
       </c>
       <c r="C156" s="2" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:4">
       <c r="A157" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B157" s="27" t="s">
+      <c r="B157" s="34" t="s">
         <v>237</v>
       </c>
       <c r="C157" s="2" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:4">
       <c r="A158" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B158" s="27" t="s">
+      <c r="B158" s="34" t="s">
         <v>239</v>
       </c>
       <c r="C158" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:4">
       <c r="A159" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B159" s="27">
+      <c r="B159" s="34">
         <v>436</v>
       </c>
       <c r="C159" s="2" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:4">
       <c r="A161" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B161" s="27">
+      <c r="B161" s="34">
         <v>437</v>
       </c>
       <c r="C161" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:4">
       <c r="A162" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B162" s="27">
+      <c r="B162" s="34">
         <v>438</v>
       </c>
       <c r="C162" s="2" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:4">
       <c r="A163" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B163" s="27">
+      <c r="B163" s="34">
         <v>438</v>
       </c>
       <c r="C163" s="2" t="s">
@@ -4223,132 +4220,132 @@
         <v>244</v>
       </c>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:4">
       <c r="A164" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B164" s="27">
+      <c r="B164" s="34">
         <v>499</v>
       </c>
       <c r="C164" s="2" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:4">
       <c r="A166" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B166" s="27">
+      <c r="B166" s="34">
         <v>440</v>
       </c>
       <c r="C166" s="2" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:4">
       <c r="A167" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B167" s="27">
+      <c r="B167" s="34">
         <v>440</v>
       </c>
       <c r="C167" s="23" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:4">
       <c r="A168" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B168" s="27" t="s">
+      <c r="B168" s="34" t="s">
         <v>248</v>
       </c>
       <c r="C168" s="2" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:4">
       <c r="A169" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B169" s="27" t="s">
+      <c r="B169" s="34" t="s">
         <v>250</v>
       </c>
       <c r="C169" s="2" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:4">
       <c r="A170" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B170" s="27">
+      <c r="B170" s="34">
         <v>444</v>
       </c>
       <c r="C170" s="2" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:4">
       <c r="A171" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B171" s="27">
+      <c r="B171" s="34">
         <v>445</v>
       </c>
       <c r="C171" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:4">
       <c r="A172" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B172" s="27">
+      <c r="B172" s="34">
         <v>447</v>
       </c>
       <c r="C172" s="2" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:4">
       <c r="A173" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B173" s="27">
+      <c r="B173" s="34">
         <v>447</v>
       </c>
       <c r="C173" s="2" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:4">
       <c r="A174" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B174" s="27">
+      <c r="B174" s="34">
         <v>447</v>
       </c>
       <c r="C174" s="2" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:4">
       <c r="A175" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B175" s="27">
+      <c r="B175" s="34">
         <v>448</v>
       </c>
       <c r="C175" s="2" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:4">
       <c r="A176" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B176" s="27">
+      <c r="B176" s="34">
         <v>488</v>
       </c>
       <c r="C176" s="2" t="s">
@@ -4358,176 +4355,176 @@
         <v>258</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3">
       <c r="A178" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B178" s="27">
+      <c r="B178" s="34">
         <v>449</v>
       </c>
       <c r="C178" s="2" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3">
       <c r="A179" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B179" s="27">
+      <c r="B179" s="34">
         <v>449</v>
       </c>
       <c r="C179" s="2" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3">
       <c r="A180" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B180" s="27">
+      <c r="B180" s="34">
         <v>449</v>
       </c>
       <c r="C180" s="2" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3">
       <c r="A181" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B181" s="27">
+      <c r="B181" s="34">
         <v>449</v>
       </c>
       <c r="C181" s="2" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3">
       <c r="A182" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B182" s="27">
+      <c r="B182" s="34">
         <v>449</v>
       </c>
       <c r="C182" s="2" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3">
       <c r="A183" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B183" s="27">
+      <c r="B183" s="34">
         <v>449</v>
       </c>
       <c r="C183" s="2" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3">
       <c r="A184" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B184" s="27" t="s">
+      <c r="B184" s="34" t="s">
         <v>265</v>
       </c>
       <c r="C184" s="2" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3">
       <c r="A186" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B186" s="27">
+      <c r="B186" s="34">
         <v>451</v>
       </c>
       <c r="C186" s="2" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3">
       <c r="A187" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B187" s="27">
+      <c r="B187" s="34">
         <v>451</v>
       </c>
       <c r="C187" s="2" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3">
       <c r="A189" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B189" s="27">
+      <c r="B189" s="34">
         <v>453</v>
       </c>
       <c r="C189" s="2" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3">
       <c r="A190" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B190" s="27">
+      <c r="B190" s="34">
         <v>453</v>
       </c>
       <c r="C190" s="2" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3">
       <c r="A191" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B191" s="27" t="s">
+      <c r="B191" s="34" t="s">
         <v>271</v>
       </c>
       <c r="C191" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3">
       <c r="A192" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B192" s="27">
+      <c r="B192" s="34">
         <v>454</v>
       </c>
       <c r="C192" s="23" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:4">
       <c r="A193" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B193" s="27">
+      <c r="B193" s="34">
         <v>454</v>
       </c>
       <c r="C193" s="2" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:4">
       <c r="A194" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B194" s="27">
+      <c r="B194" s="34">
         <v>454</v>
       </c>
       <c r="C194" s="2" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:4">
       <c r="A195" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B195" s="27">
+      <c r="B195" s="34">
         <v>455</v>
       </c>
       <c r="C195" s="2" t="s">
@@ -4537,172 +4534,172 @@
         <v>276</v>
       </c>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:4">
       <c r="A197" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B197" s="27">
+      <c r="B197" s="34">
         <v>456</v>
       </c>
       <c r="C197" s="2" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:4">
       <c r="A198" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B198" s="27" t="s">
+      <c r="B198" s="34" t="s">
         <v>278</v>
       </c>
       <c r="C198" s="23" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:4">
       <c r="A199" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B199" s="27">
+      <c r="B199" s="34">
         <v>458</v>
       </c>
       <c r="C199" s="2" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:4">
       <c r="A200" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B200" s="27">
+      <c r="B200" s="34">
         <v>459</v>
       </c>
       <c r="C200" s="2" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:4">
       <c r="A202" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B202" s="27">
+      <c r="B202" s="34">
         <v>460</v>
       </c>
       <c r="C202" s="2" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:4">
       <c r="A203" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B203" s="27">
+      <c r="B203" s="34">
         <v>462</v>
       </c>
       <c r="C203" s="2" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:4">
       <c r="A205" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B205" s="27">
+      <c r="B205" s="34">
         <v>463</v>
       </c>
       <c r="C205" s="2" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:4">
       <c r="A206" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B206" s="27">
+      <c r="B206" s="34">
         <v>463</v>
       </c>
       <c r="C206" s="2" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:4">
       <c r="A207" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B207" s="27">
+      <c r="B207" s="34">
         <v>465</v>
       </c>
       <c r="C207" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:4">
       <c r="A208" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="B208" s="27">
+      <c r="B208" s="34">
         <v>467</v>
       </c>
       <c r="C208" s="23" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:4">
       <c r="A209" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B209" s="27" t="s">
+      <c r="B209" s="34" t="s">
         <v>288</v>
       </c>
       <c r="C209" s="23" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:4">
       <c r="A210" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B210" s="27">
+      <c r="B210" s="34">
         <v>468</v>
       </c>
       <c r="C210" s="2" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:4">
       <c r="A211" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B211" s="27" t="s">
+      <c r="B211" s="34" t="s">
         <v>291</v>
       </c>
       <c r="C211" s="2" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:4">
       <c r="A212" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B212" s="27">
+      <c r="B212" s="34">
         <v>470</v>
       </c>
       <c r="C212" s="2" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:4">
       <c r="A213" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B213" s="27">
+      <c r="B213" s="34">
         <v>472</v>
       </c>
       <c r="C213" s="2" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:4">
       <c r="A214" s="1" t="s">
         <v>295</v>
       </c>
@@ -4713,44 +4710,44 @@
         <v>297</v>
       </c>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:4">
       <c r="A215" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B215" s="27" t="s">
+      <c r="B215" s="34" t="s">
         <v>298</v>
       </c>
       <c r="C215" s="23" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:4">
       <c r="A217" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B217" s="27">
+      <c r="B217" s="34">
         <v>480</v>
       </c>
       <c r="C217" s="2" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:4">
       <c r="A218" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B218" s="27">
+      <c r="B218" s="34">
         <v>482</v>
       </c>
       <c r="C218" s="2" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:4">
       <c r="A220" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B220" s="27">
+      <c r="B220" s="34">
         <v>484</v>
       </c>
       <c r="C220" s="2" t="s">
@@ -4760,22 +4757,22 @@
         <v>78</v>
       </c>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:4">
       <c r="A221" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B221" s="27">
+      <c r="B221" s="34">
         <v>486</v>
       </c>
       <c r="C221" s="2" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:4">
       <c r="A222" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B222" s="27">
+      <c r="B222" s="34">
         <v>486</v>
       </c>
       <c r="C222" s="2" t="s">
@@ -4785,7 +4782,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:4">
       <c r="A223" s="1" t="s">
         <v>5</v>
       </c>

</xml_diff>